<commit_message>
Fix scale-parsing bug in account counts, restore MS Legacy tier, anchor KPIs to latest year, pin deps
</commit_message>
<xml_diff>
--- a/samples/CSPN_Prepaid_Consolidated_2005-2025.xlsx
+++ b/samples/CSPN_Prepaid_Consolidated_2005-2025.xlsx
@@ -538,7 +538,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Generated by the Prepaid Committee Data Tool on 2026-07-12. One row per plan per reporting period.</t>
+          <t>Generated by the Prepaid Committee Data Tool on 2026-07-13. One row per plan per reporting period.</t>
         </is>
       </c>
     </row>
@@ -2010,7 +2010,7 @@
         <v>535791</v>
       </c>
       <c r="I34" s="8" t="n">
-        <v>1</v>
+        <v>1370000</v>
       </c>
       <c r="J34" s="7" t="n">
         <v>287</v>
@@ -2059,7 +2059,7 @@
         <v>502938</v>
       </c>
       <c r="I35" s="8" t="n">
-        <v>1</v>
+        <v>1370000</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>359</v>
@@ -2703,7 +2703,7 @@
         <v>5044</v>
       </c>
       <c r="I51" s="8" t="n">
-        <v>44</v>
+        <v>44000</v>
       </c>
       <c r="J51" s="7" t="n">
         <v>6</v>
@@ -2752,7 +2752,7 @@
         <v>5081</v>
       </c>
       <c r="I52" s="8" t="n">
-        <v>44</v>
+        <v>44000</v>
       </c>
       <c r="J52" s="7" t="n">
         <v>7.1</v>
@@ -2801,7 +2801,7 @@
         <v>4733</v>
       </c>
       <c r="I53" s="8" t="n">
-        <v>45</v>
+        <v>45000</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>9.1</v>
@@ -4289,7 +4289,7 @@
       </c>
       <c r="M88" s="5" t="inlineStr">
         <is>
-          <t>MET II (Plan D)</t>
+          <t>MET II (Plan D); All data is as of 9/30/25</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,11 @@
           <t>CSPN Prepaid Committee Fall 2025</t>
         </is>
       </c>
-      <c r="M105" s="5" t="n"/>
+      <c r="M105" s="5" t="inlineStr">
+        <is>
+          <t>Legacy tier 106%</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
@@ -9647,7 +9651,7 @@
       </c>
       <c r="M212" s="5" t="inlineStr">
         <is>
-          <t>MET I (Plans B &amp; C)</t>
+          <t>MET I (Plans B &amp; C); All data is as of 9/30/25</t>
         </is>
       </c>
     </row>

</xml_diff>